<commit_message>
ajuste na meta do televendas . filial 7
</commit_message>
<xml_diff>
--- a/data/meta_televendas.xlsx
+++ b/data/meta_televendas.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\christian.roque\Desktop\Total_Day\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{082D187D-4177-4474-8FF9-5376A6EDB674}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33B471A8-D049-4135-A889-92D4B75875D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,16 +46,23 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="_-[$R$-416]\ * #,##0.00_-;\-[$R$-416]\ * #,##0.00_-;_-[$R$-416]\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="&quot;R$&quot;\ #,##0.00;[Red]\-&quot;R$&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -75,10 +82,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -86,9 +94,16 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{FB098738-3403-4C67-B238-0CFE129E26F1}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -391,7 +406,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.44140625" bestFit="1" customWidth="1"/>
@@ -828,6 +843,105 @@
         <v>66661.805334142555</v>
       </c>
     </row>
+    <row r="40" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A40" s="1">
+        <v>7</v>
+      </c>
+      <c r="B40" s="3">
+        <v>519</v>
+      </c>
+      <c r="C40" s="4">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A41" s="1">
+        <v>7</v>
+      </c>
+      <c r="B41" s="3">
+        <v>1883</v>
+      </c>
+      <c r="C41" s="4">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A42" s="1">
+        <v>7</v>
+      </c>
+      <c r="B42" s="3">
+        <v>1885</v>
+      </c>
+      <c r="C42" s="4">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A43" s="1">
+        <v>7</v>
+      </c>
+      <c r="B43" s="3">
+        <v>1899</v>
+      </c>
+      <c r="C43" s="4">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A44" s="1">
+        <v>7</v>
+      </c>
+      <c r="B44" s="3">
+        <v>2184</v>
+      </c>
+      <c r="C44" s="4">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A45" s="1">
+        <v>7</v>
+      </c>
+      <c r="B45" s="3">
+        <v>1884</v>
+      </c>
+      <c r="C45" s="4">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A46" s="1">
+        <v>7</v>
+      </c>
+      <c r="B46" s="3">
+        <v>2185</v>
+      </c>
+      <c r="C46" s="4">
+        <v>33333</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A47" s="1">
+        <v>7</v>
+      </c>
+      <c r="B47" s="3">
+        <v>3389</v>
+      </c>
+      <c r="C47" s="4">
+        <v>33333</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A48" s="1">
+        <v>7</v>
+      </c>
+      <c r="B48" s="3">
+        <v>2985</v>
+      </c>
+      <c r="C48" s="4">
+        <v>33334</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>